<commit_message>
updated os24 squamous subanalysis mlef
</commit_message>
<xml_diff>
--- a/mlef_pipeline/results/OS_24/SQUAMOUS/RWD/results.xlsx
+++ b/mlef_pipeline/results/OS_24/SQUAMOUS/RWD/results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,22 +468,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0.64 ± 0.09</t>
+          <t>0.64 ± 0.08</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.43 ± 0.11</t>
+          <t>0.44 ± 0.07</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.62 ± 0.24</t>
+          <t>0.51 ± 0.20</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.48 ± 0.17</t>
+          <t>0.55 ± 0.16</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -498,22 +498,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.67 ± 0.17</t>
+          <t>0.75 ± 0.16</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.53</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.28</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -528,22 +528,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.81 ± 0.19</t>
+          <t>0.62 ± 0.33</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.74</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.80</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.69</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="F4" t="n">

</xml_diff>